<commit_message>
fix: move data.xlsx to public folder for build script
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xueruifang/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xueruifang/Desktop/手搓我的Sims世界/sims-files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B762A0-3739-D044-B7AA-13C00DB57A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8354D9D-4B65-DE46-9552-205DC9957E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="368">
   <si>
     <t>id</t>
   </si>
@@ -114,36 +114,39 @@
     <t>FALSE</t>
   </si>
   <si>
+    <t>Creative,Bookworm,Outgoing</t>
+  </si>
+  <si>
+    <t>Bestselling Author</t>
+  </si>
+  <si>
+    <t>Writing:8,Logic:6,Charisma:5</t>
+  </si>
+  <si>
+    <t>GothBella</t>
+  </si>
+  <si>
+    <t>GothCassandra,GothAlexander</t>
+  </si>
+  <si>
+    <t>GothGunther,GothCornelia</t>
+  </si>
+  <si>
+    <t>Bella Goth</t>
+  </si>
+  <si>
+    <t>贝拉·哥特</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Secret Agent</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Bestselling Author</t>
-  </si>
-  <si>
-    <t>Writing:8,Logic:6,Charisma:5</t>
-  </si>
-  <si>
-    <t>GothBella</t>
-  </si>
-  <si>
-    <t>GothCassandra,GothAlexander</t>
-  </si>
-  <si>
-    <t>GothGunther,GothCornelia</t>
-  </si>
-  <si>
-    <t>Bella Goth</t>
-  </si>
-  <si>
-    <t>贝拉·哥特</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Secret Agent</t>
-  </si>
-  <si>
     <t>GothCassandra</t>
   </si>
   <si>
@@ -162,9 +165,6 @@
     <t>High School Student</t>
   </si>
   <si>
-    <t>Violin:1</t>
-  </si>
-  <si>
     <t>GothAlexander</t>
   </si>
   <si>
@@ -180,9 +180,6 @@
     <t>Grade School Student</t>
   </si>
   <si>
-    <t>Creativity:1</t>
-  </si>
-  <si>
     <t>KimDennis</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>Retired</t>
   </si>
   <si>
-    <t>Gardening:1</t>
-  </si>
-  <si>
     <t>SpencerLydia</t>
   </si>
   <si>
@@ -225,9 +219,6 @@
     <t>Business</t>
   </si>
   <si>
-    <t>Logic:1</t>
-  </si>
-  <si>
     <t>SpencerKimAlice</t>
   </si>
   <si>
@@ -246,9 +237,6 @@
     <t>Painter</t>
   </si>
   <si>
-    <t>Painting:1</t>
-  </si>
-  <si>
     <t>LewisEric</t>
   </si>
   <si>
@@ -261,9 +249,6 @@
     <t>Tech Guru</t>
   </si>
   <si>
-    <t>Programming:1</t>
-  </si>
-  <si>
     <t>KimLewisOlivia</t>
   </si>
   <si>
@@ -273,9 +258,6 @@
     <t>奥利维亚·金-刘易斯</t>
   </si>
   <si>
-    <t>Motor:1</t>
-  </si>
-  <si>
     <t>PancakesBob</t>
   </si>
   <si>
@@ -291,9 +273,6 @@
     <t>Culinary</t>
   </si>
   <si>
-    <t>Cooking:1</t>
-  </si>
-  <si>
     <t>PancakesEliza</t>
   </si>
   <si>
@@ -306,9 +285,6 @@
     <t>Unemployed</t>
   </si>
   <si>
-    <t>Fitness:1</t>
-  </si>
-  <si>
     <t>HolidaySummer</t>
   </si>
   <si>
@@ -333,9 +309,6 @@
     <t>特拉维斯·斯科特</t>
   </si>
   <si>
-    <t>Video Gaming:1</t>
-  </si>
-  <si>
     <t>LeeLiberty</t>
   </si>
   <si>
@@ -351,9 +324,6 @@
     <t>Astronaut</t>
   </si>
   <si>
-    <t>Rocket Science:1</t>
-  </si>
-  <si>
     <t>description</t>
   </si>
   <si>
@@ -786,316 +756,382 @@
     <t>GreenLlama</t>
   </si>
   <si>
+    <t>Male Hair,Female Hair,Clothes</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>https://patreon.com</t>
+  </si>
+  <si>
+    <t>peacemaker</t>
+  </si>
+  <si>
+    <t>Peacemaker</t>
+  </si>
+  <si>
+    <t>Furniture,Build Items</t>
+  </si>
+  <si>
+    <t>sentate</t>
+  </si>
+  <si>
+    <t>Sentate</t>
+  </si>
+  <si>
+    <t>Clothes,Shoes</t>
+  </si>
+  <si>
+    <t>aharris00britney</t>
+  </si>
+  <si>
+    <t>Aharris00britney</t>
+  </si>
+  <si>
+    <t>Female Hair,Clothes</t>
+  </si>
+  <si>
+    <t>felixandre</t>
+  </si>
+  <si>
+    <t>Felixandre</t>
+  </si>
+  <si>
+    <t>harrie</t>
+  </si>
+  <si>
+    <t>Harrie</t>
+  </si>
+  <si>
+    <t>simstrouble</t>
+  </si>
+  <si>
+    <t>SimsTrouble</t>
+  </si>
+  <si>
+    <t>Female Hair</t>
+  </si>
+  <si>
+    <t>johnnysims</t>
+  </si>
+  <si>
+    <t>Johnnysims</t>
+  </si>
+  <si>
+    <t>Male Hair</t>
+  </si>
+  <si>
+    <t>rusty</t>
+  </si>
+  <si>
+    <t>Rusty</t>
+  </si>
+  <si>
+    <t>Clothes,Male Hair</t>
+  </si>
+  <si>
+    <t>Not Updating</t>
+  </si>
+  <si>
+    <t>clumsyalien</t>
+  </si>
+  <si>
+    <t>ClumsyAlien</t>
+  </si>
+  <si>
+    <t>Clothes,Female Hair</t>
+  </si>
+  <si>
+    <t>twistedmexi</t>
+  </si>
+  <si>
+    <t>TwistedMexi</t>
+  </si>
+  <si>
+    <t>Mods,Build Items</t>
+  </si>
+  <si>
+    <t>lumpinou</t>
+  </si>
+  <si>
+    <t>Lumpinou</t>
+  </si>
+  <si>
+    <t>Mods,Gameplay</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>author</t>
+  </si>
+  <si>
+    <t>subtype</t>
+  </si>
+  <si>
+    <t>translationUrl</t>
+  </si>
+  <si>
+    <t>goth-galore-hair</t>
+  </si>
+  <si>
+    <t>Goth Galore Hair</t>
+  </si>
+  <si>
+    <t>CAS</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>mid-century-modern-sofa</t>
+  </si>
+  <si>
+    <t>Mid-Century Modern Sofa</t>
+  </si>
+  <si>
+    <t>Build/Buy</t>
+  </si>
+  <si>
+    <t>Furniture</t>
+  </si>
+  <si>
+    <t>better-buildbuy</t>
+  </si>
+  <si>
+    <t>Better BuildBuy</t>
+  </si>
+  <si>
+    <t>Mods</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>woohoo-wellness</t>
+  </si>
+  <si>
+    <t>WooHoo Wellness</t>
+  </si>
+  <si>
+    <t>Gameplay</t>
+  </si>
+  <si>
+    <t>vintage-glamour-dress</t>
+  </si>
+  <si>
+    <t>Vintage Glamour Dress</t>
+  </si>
+  <si>
+    <t>Clothes</t>
+  </si>
+  <si>
+    <t>rustic-kitchen-counters</t>
+  </si>
+  <si>
+    <t>Rustic Kitchen Counters</t>
+  </si>
+  <si>
+    <t>chunky-boots</t>
+  </si>
+  <si>
+    <t>Chunky Boots</t>
+  </si>
+  <si>
+    <t>Shoes</t>
+  </si>
+  <si>
+    <t>messy-male-hair</t>
+  </si>
+  <si>
+    <t>Messy Male Hair</t>
+  </si>
+  <si>
+    <t>mc-command-center</t>
+  </si>
+  <si>
+    <t>MC Command Center</t>
+  </si>
+  <si>
+    <t>Deaderpool</t>
+  </si>
+  <si>
+    <t>Core</t>
+  </si>
+  <si>
+    <t>boho-bedroom-set</t>
+  </si>
+  <si>
+    <t>Boho Bedroom Set</t>
+  </si>
+  <si>
+    <t>maxis-match-cc-world</t>
+  </si>
+  <si>
+    <t>Maxis Match CC World</t>
+  </si>
+  <si>
+    <t>https://maxismatchccworld.tumblr.com/</t>
+  </si>
+  <si>
+    <t>snootysims</t>
+  </si>
+  <si>
+    <t>SnootySims</t>
+  </si>
+  <si>
+    <t>https://snootysims.com/</t>
+  </si>
+  <si>
+    <t>the-sims-resource</t>
+  </si>
+  <si>
+    <t>The Sims Resource</t>
+  </si>
+  <si>
+    <t>https://www.thesimsresource.com/</t>
+  </si>
+  <si>
+    <t>mod-the-sims</t>
+  </si>
+  <si>
+    <t>Mod The Sims</t>
+  </si>
+  <si>
+    <t>https://modthesims.info/</t>
+  </si>
+  <si>
+    <t>sims-4-updates</t>
+  </si>
+  <si>
+    <t>Sims 4 Updates</t>
+  </si>
+  <si>
+    <t>https://sims4updates.net/</t>
+  </si>
+  <si>
+    <t>lilsimsie-cc-finds</t>
+  </si>
+  <si>
+    <t>Lilsimsie CC Finds</t>
+  </si>
+  <si>
+    <t>https://lilsimsiecc.tumblr.com/</t>
+  </si>
+  <si>
+    <t>gal1</t>
+  </si>
+  <si>
+    <t>gal2</t>
+  </si>
+  <si>
+    <t>gal3</t>
+  </si>
+  <si>
+    <t>gal4</t>
+  </si>
+  <si>
+    <t>gal5</t>
+  </si>
+  <si>
+    <t>gal6</t>
+  </si>
+  <si>
+    <t>gal7</t>
+  </si>
+  <si>
+    <t>gal8</t>
+  </si>
+  <si>
+    <t>gal9</t>
+  </si>
+  <si>
+    <t>gal10</t>
+  </si>
+  <si>
+    <t>gal11</t>
+  </si>
+  <si>
+    <t>gal12</t>
+  </si>
+  <si>
+    <t>haha</t>
+  </si>
+  <si>
+    <t>dss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dsfes </t>
+  </si>
+  <si>
+    <t>fangfang</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t xml:space="preserve">single </t>
+  </si>
+  <si>
+    <t>Teacher</t>
+  </si>
+  <si>
+    <t>FANGFFF</t>
+  </si>
+  <si>
+    <t>BLOOMS</t>
+  </si>
+  <si>
+    <t>32x32</t>
+  </si>
+  <si>
+    <t>SmallBusiness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zhuzhu </t>
+  </si>
+  <si>
+    <t>zhuzhu</t>
+  </si>
+  <si>
+    <t>女发</t>
+  </si>
+  <si>
+    <t xml:space="preserve">编织:2, 钢琴:2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCCC </t>
+  </si>
+  <si>
+    <t>B必备</t>
+  </si>
+  <si>
+    <t>AAA必备</t>
+  </si>
+  <si>
+    <t>blooms</t>
+  </si>
+  <si>
+    <t>lovestuck</t>
+  </si>
+  <si>
+    <t>Lovestuck</t>
+  </si>
+  <si>
+    <t>恋爱之城</t>
+  </si>
+  <si>
     <t>A</t>
   </si>
   <si>
-    <t>Male Hair,Female Hair,Clothes</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>https://patreon.com</t>
-  </si>
-  <si>
-    <t>peacemaker</t>
-  </si>
-  <si>
-    <t>Peacemaker</t>
-  </si>
-  <si>
-    <t>Furniture,Build Items</t>
-  </si>
-  <si>
-    <t>sentate</t>
-  </si>
-  <si>
-    <t>Sentate</t>
-  </si>
-  <si>
-    <t>Clothes,Shoes</t>
-  </si>
-  <si>
-    <t>aharris00britney</t>
-  </si>
-  <si>
-    <t>Aharris00britney</t>
-  </si>
-  <si>
-    <t>Female Hair,Clothes</t>
-  </si>
-  <si>
-    <t>felixandre</t>
-  </si>
-  <si>
-    <t>Felixandre</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>harrie</t>
-  </si>
-  <si>
-    <t>Harrie</t>
-  </si>
-  <si>
-    <t>simstrouble</t>
-  </si>
-  <si>
-    <t>SimsTrouble</t>
-  </si>
-  <si>
-    <t>Female Hair</t>
-  </si>
-  <si>
-    <t>johnnysims</t>
-  </si>
-  <si>
-    <t>Johnnysims</t>
-  </si>
-  <si>
-    <t>Male Hair</t>
-  </si>
-  <si>
-    <t>rusty</t>
-  </si>
-  <si>
-    <t>Rusty</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>Clothes,Male Hair</t>
-  </si>
-  <si>
-    <t>Not Updating</t>
-  </si>
-  <si>
-    <t>clumsyalien</t>
-  </si>
-  <si>
-    <t>ClumsyAlien</t>
-  </si>
-  <si>
-    <t>Clothes,Female Hair</t>
-  </si>
-  <si>
-    <t>twistedmexi</t>
-  </si>
-  <si>
-    <t>TwistedMexi</t>
-  </si>
-  <si>
-    <t>Mods,Build Items</t>
-  </si>
-  <si>
-    <t>lumpinou</t>
-  </si>
-  <si>
-    <t>Lumpinou</t>
-  </si>
-  <si>
-    <t>Mods,Gameplay</t>
-  </si>
-  <si>
-    <t>title</t>
-  </si>
-  <si>
-    <t>author</t>
-  </si>
-  <si>
-    <t>subtype</t>
-  </si>
-  <si>
-    <t>translationUrl</t>
-  </si>
-  <si>
-    <t>goth-galore-hair</t>
-  </si>
-  <si>
-    <t>Goth Galore Hair</t>
-  </si>
-  <si>
-    <t>CAS</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>mid-century-modern-sofa</t>
-  </si>
-  <si>
-    <t>Mid-Century Modern Sofa</t>
-  </si>
-  <si>
-    <t>Build/Buy</t>
-  </si>
-  <si>
-    <t>Furniture</t>
-  </si>
-  <si>
-    <t>better-buildbuy</t>
-  </si>
-  <si>
-    <t>Better BuildBuy</t>
-  </si>
-  <si>
-    <t>Mods</t>
-  </si>
-  <si>
-    <t>UI</t>
-  </si>
-  <si>
-    <t>woohoo-wellness</t>
-  </si>
-  <si>
-    <t>WooHoo Wellness</t>
-  </si>
-  <si>
-    <t>Gameplay</t>
-  </si>
-  <si>
-    <t>vintage-glamour-dress</t>
-  </si>
-  <si>
-    <t>Vintage Glamour Dress</t>
-  </si>
-  <si>
-    <t>Clothes</t>
-  </si>
-  <si>
-    <t>rustic-kitchen-counters</t>
-  </si>
-  <si>
-    <t>Rustic Kitchen Counters</t>
-  </si>
-  <si>
-    <t>chunky-boots</t>
-  </si>
-  <si>
-    <t>Chunky Boots</t>
-  </si>
-  <si>
-    <t>Shoes</t>
-  </si>
-  <si>
-    <t>messy-male-hair</t>
-  </si>
-  <si>
-    <t>Messy Male Hair</t>
-  </si>
-  <si>
-    <t>mc-command-center</t>
-  </si>
-  <si>
-    <t>MC Command Center</t>
-  </si>
-  <si>
-    <t>Deaderpool</t>
-  </si>
-  <si>
-    <t>Core</t>
-  </si>
-  <si>
-    <t>boho-bedroom-set</t>
-  </si>
-  <si>
-    <t>Boho Bedroom Set</t>
-  </si>
-  <si>
-    <t>maxis-match-cc-world</t>
-  </si>
-  <si>
-    <t>Maxis Match CC World</t>
-  </si>
-  <si>
-    <t>https://maxismatchccworld.tumblr.com/</t>
-  </si>
-  <si>
-    <t>snootysims</t>
-  </si>
-  <si>
-    <t>SnootySims</t>
-  </si>
-  <si>
-    <t>https://snootysims.com/</t>
-  </si>
-  <si>
-    <t>the-sims-resource</t>
-  </si>
-  <si>
-    <t>The Sims Resource</t>
-  </si>
-  <si>
-    <t>https://www.thesimsresource.com/</t>
-  </si>
-  <si>
-    <t>mod-the-sims</t>
-  </si>
-  <si>
-    <t>Mod The Sims</t>
-  </si>
-  <si>
-    <t>https://modthesims.info/</t>
-  </si>
-  <si>
-    <t>sims-4-updates</t>
-  </si>
-  <si>
-    <t>Sims 4 Updates</t>
-  </si>
-  <si>
-    <t>https://sims4updates.net/</t>
-  </si>
-  <si>
-    <t>lilsimsie-cc-finds</t>
-  </si>
-  <si>
-    <t>Lilsimsie CC Finds</t>
-  </si>
-  <si>
-    <t>https://lilsimsiecc.tumblr.com/</t>
-  </si>
-  <si>
-    <t>gal1</t>
-  </si>
-  <si>
-    <t>gal2</t>
-  </si>
-  <si>
-    <t>gal3</t>
-  </si>
-  <si>
-    <t>gal4</t>
-  </si>
-  <si>
-    <t>gal5</t>
-  </si>
-  <si>
-    <t>gal6</t>
-  </si>
-  <si>
-    <t>gal7</t>
-  </si>
-  <si>
-    <t>gal8</t>
-  </si>
-  <si>
-    <t>gal9</t>
-  </si>
-  <si>
-    <t>gal10</t>
-  </si>
-  <si>
-    <t>gal11</t>
-  </si>
-  <si>
-    <t>gal12</t>
-  </si>
-  <si>
-    <t>Charisma:1,</t>
+    <t>mccc</t>
+  </si>
+  <si>
+    <t>fangcc</t>
   </si>
 </sst>
 </file>
@@ -1472,11 +1508,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="14" max="14" width="45.6640625" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1619,45 +1652,45 @@
         <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N3" t="s">
-        <v>355</v>
+        <v>38</v>
       </c>
       <c r="O3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
         <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H4" t="s">
         <v>24</v>
@@ -1666,28 +1699,28 @@
         <v>25</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K4" t="s">
         <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="O4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -1710,7 +1743,7 @@
         <v>48</v>
       </c>
       <c r="G5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H5" t="s">
         <v>24</v>
@@ -1725,45 +1758,45 @@
         <v>27</v>
       </c>
       <c r="L5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N5" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="O5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
         <v>51</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>52</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>53</v>
-      </c>
-      <c r="D6" t="s">
-        <v>54</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" t="s">
         <v>55</v>
-      </c>
-      <c r="G6" t="s">
-        <v>56</v>
       </c>
       <c r="H6" t="s">
         <v>24</v>
@@ -1772,42 +1805,42 @@
         <v>25</v>
       </c>
       <c r="J6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K6" t="s">
         <v>27</v>
       </c>
       <c r="L6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N6" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="O6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
         <v>59</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>60</v>
-      </c>
-      <c r="C7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" t="s">
-        <v>62</v>
       </c>
       <c r="E7" t="s">
         <v>36</v>
@@ -1816,7 +1849,7 @@
         <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H7" t="s">
         <v>24</v>
@@ -1825,48 +1858,48 @@
         <v>25</v>
       </c>
       <c r="J7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K7" t="s">
         <v>27</v>
       </c>
       <c r="L7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N7" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="O7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" t="s">
         <v>66</v>
-      </c>
-      <c r="B8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" t="s">
-        <v>69</v>
       </c>
       <c r="E8" t="s">
         <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G8" t="s">
         <v>23</v>
@@ -1878,48 +1911,48 @@
         <v>25</v>
       </c>
       <c r="J8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="K8" t="s">
         <v>27</v>
       </c>
       <c r="L8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N8" t="s">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="O8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E9" t="s">
         <v>21</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G9" t="s">
         <v>23</v>
@@ -1931,42 +1964,42 @@
         <v>25</v>
       </c>
       <c r="J9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="K9" t="s">
         <v>27</v>
       </c>
       <c r="L9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N9" t="s">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="O9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E10" t="s">
         <v>36</v>
@@ -1975,7 +2008,7 @@
         <v>48</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H10" t="s">
         <v>24</v>
@@ -1990,42 +2023,42 @@
         <v>27</v>
       </c>
       <c r="L10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N10" t="s">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="O10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E11" t="s">
         <v>21</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
         <v>23</v>
@@ -2037,48 +2070,48 @@
         <v>25</v>
       </c>
       <c r="J11" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K11" t="s">
         <v>27</v>
       </c>
       <c r="L11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N11" t="s">
-        <v>87</v>
+        <v>38</v>
       </c>
       <c r="O11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" t="s">
         <v>83</v>
-      </c>
-      <c r="C12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D12" t="s">
-        <v>90</v>
       </c>
       <c r="E12" t="s">
         <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G12" t="s">
         <v>23</v>
@@ -2090,51 +2123,51 @@
         <v>25</v>
       </c>
       <c r="J12" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="K12" t="s">
         <v>27</v>
       </c>
       <c r="L12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N12" t="s">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="O12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="E13" t="s">
         <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H13" t="s">
         <v>24</v>
@@ -2143,51 +2176,51 @@
         <v>25</v>
       </c>
       <c r="J13" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K13" t="s">
         <v>27</v>
       </c>
       <c r="L13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N13" t="s">
-        <v>87</v>
+        <v>38</v>
       </c>
       <c r="O13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="E14" t="s">
         <v>21</v>
       </c>
       <c r="F14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H14" t="s">
         <v>24</v>
@@ -2196,51 +2229,51 @@
         <v>25</v>
       </c>
       <c r="J14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="K14" t="s">
         <v>27</v>
       </c>
       <c r="L14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N14" t="s">
-        <v>101</v>
+        <v>38</v>
       </c>
       <c r="O14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="D15" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="E15" t="s">
         <v>36</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H15" t="s">
         <v>24</v>
@@ -2249,41 +2282,79 @@
         <v>25</v>
       </c>
       <c r="J15" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="K15" t="s">
         <v>27</v>
       </c>
       <c r="L15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="M15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="N15" t="s">
-        <v>107</v>
+        <v>38</v>
       </c>
       <c r="O15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="P15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="Q15" t="s">
-        <v>28</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>342</v>
+      </c>
+      <c r="B16" t="s">
+        <v>343</v>
+      </c>
+      <c r="C16" t="s">
+        <v>344</v>
+      </c>
+      <c r="D16" t="s">
+        <v>345</v>
+      </c>
+      <c r="E16" t="s">
+        <v>346</v>
+      </c>
+      <c r="F16" t="s">
+        <v>347</v>
+      </c>
+      <c r="G16" t="s">
+        <v>348</v>
+      </c>
+      <c r="H16" t="s">
+        <v>119</v>
+      </c>
+      <c r="I16" t="s">
+        <v>120</v>
+      </c>
+      <c r="J16" t="s">
+        <v>349</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="N16" t="s">
+        <v>357</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:Q2 A4:Q15 A3:M3 O3:Q3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K15 L1:Q15" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -2297,7 +2368,7 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E1" t="s">
         <v>7</v>
@@ -2306,13 +2377,13 @@
         <v>8</v>
       </c>
       <c r="G1" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H1" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="I1" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -2320,13 +2391,13 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E2" t="s">
         <v>24</v>
@@ -2335,27 +2406,27 @@
         <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="H2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="I2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
         <v>24</v>
@@ -2364,27 +2435,27 @@
         <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="H3" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="I3" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
         <v>24</v>
@@ -2393,27 +2464,27 @@
         <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="B5" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
         <v>24</v>
@@ -2422,303 +2493,317 @@
         <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="F6" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B7" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="F7" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="F8" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="F9" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="G9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B10" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="F10" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="G10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B11" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E11" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="F11" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="G11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="F12" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="G12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="F13" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="G13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="F14" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="G14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="B15" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E15" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="F15" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="G15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I15" t="s">
-        <v>28</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>345</v>
+      </c>
+      <c r="B16" t="s">
+        <v>350</v>
+      </c>
+      <c r="E16" t="s">
+        <v>139</v>
+      </c>
+      <c r="F16" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -2731,7 +2816,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -2745,48 +2830,48 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="E1" t="s">
         <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="G1" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="H1" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="I1" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B2" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="E2" t="s">
         <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="G2" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I2" t="s">
         <v>27</v>
@@ -2794,28 +2879,28 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="B3" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E3" t="s">
         <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="G3" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I3" t="s">
         <v>27</v>
@@ -2823,28 +2908,28 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B4" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E4" t="s">
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I4" t="s">
         <v>27</v>
@@ -2852,28 +2937,28 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E5" t="s">
         <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="G5" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I5" t="s">
         <v>27</v>
@@ -2881,28 +2966,28 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="B6" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E6" t="s">
         <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G6" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I6" t="s">
         <v>27</v>
@@ -2910,28 +2995,28 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B7" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E7" t="s">
         <v>25</v>
       </c>
       <c r="F7" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G7" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I7" t="s">
         <v>27</v>
@@ -2939,28 +3024,28 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="B8" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E8" t="s">
         <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G8" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I8" t="s">
         <v>27</v>
@@ -2968,28 +3053,28 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="E9" t="s">
         <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G9" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I9" t="s">
         <v>27</v>
@@ -2997,28 +3082,28 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="B10" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="E10" t="s">
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="G10" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H10" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I10" t="s">
         <v>27</v>
@@ -3026,28 +3111,28 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="B11" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="E11" t="s">
         <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="G11" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I11" t="s">
         <v>27</v>
@@ -3055,86 +3140,86 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B12" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C12" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="D12" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="G12" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H12" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I12" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D13" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E13" t="s">
         <v>25</v>
       </c>
       <c r="F13" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G13" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H13" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I13" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="B14" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E14" t="s">
         <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G14" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="H14" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I14" t="s">
         <v>27</v>
@@ -3142,28 +3227,28 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="B15" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E15" t="s">
         <v>25</v>
       </c>
       <c r="F15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G15" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="H15" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I15" t="s">
         <v>27</v>
@@ -3171,28 +3256,28 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E16" t="s">
         <v>25</v>
       </c>
       <c r="F16" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G16" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="H16" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I16" t="s">
         <v>27</v>
@@ -3200,28 +3285,28 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B17" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="E17" t="s">
         <v>25</v>
       </c>
       <c r="F17" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G17" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="H17" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I17" t="s">
         <v>27</v>
@@ -3229,28 +3314,28 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B18" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C18" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E18" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G18" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H18" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I18" t="s">
         <v>27</v>
@@ -3258,28 +3343,28 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="B19" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E19" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F19" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G19" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H19" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I19" t="s">
         <v>27</v>
@@ -3287,28 +3372,28 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="B20" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="C20" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D20" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E20" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F20" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G20" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H20" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I20" t="s">
         <v>27</v>
@@ -3316,28 +3401,28 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B21" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D21" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E21" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F21" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G21" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H21" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I21" t="s">
         <v>27</v>
@@ -3345,28 +3430,28 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="B22" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="C22" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D22" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E22" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G22" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="H22" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I22" t="s">
         <v>27</v>
@@ -3374,28 +3459,28 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="B23" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="C23" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D23" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E23" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F23" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G23" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="H23" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I23" t="s">
         <v>27</v>
@@ -3403,28 +3488,28 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="C24" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D24" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E24" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F24" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G24" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="H24" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I24" t="s">
         <v>27</v>
@@ -3432,31 +3517,60 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="B25" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="C25" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D25" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="E25" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F25" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G25" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="H25" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I25" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>361</v>
+      </c>
+      <c r="B26" t="s">
+        <v>351</v>
+      </c>
+      <c r="C26" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" t="s">
+        <v>352</v>
+      </c>
+      <c r="E26" t="s">
+        <v>120</v>
+      </c>
+      <c r="F26" t="s">
+        <v>38</v>
+      </c>
+      <c r="G26" t="s">
+        <v>353</v>
+      </c>
+      <c r="H26" t="s">
+        <v>38</v>
+      </c>
+      <c r="I26" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3469,7 +3583,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -3483,10 +3597,10 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E1" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -3497,81 +3611,98 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="D2" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="E2" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B3" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="D3" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="E3" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="B4" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="C4" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="D4" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="E4" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C5" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="D5" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="E5" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B6" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C6" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="D6" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="E6" t="s">
-        <v>239</v>
+        <v>229</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B7" t="s">
+        <v>363</v>
+      </c>
+      <c r="C7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+      <c r="E7" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3598,7 +3729,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -3606,13 +3737,13 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C2" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="D2" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -3620,13 +3751,13 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C3" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="D3" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -3634,13 +3765,13 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="C4" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="D4" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -3653,7 +3784,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -3664,256 +3795,276 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="D1" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="E1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="F1" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
-      </c>
-      <c r="C2" t="s">
-        <v>252</v>
+        <v>241</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="E2" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F2" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
-      </c>
-      <c r="C3" t="s">
-        <v>252</v>
+        <v>246</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E3" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F3" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="B4" t="s">
-        <v>260</v>
-      </c>
-      <c r="C4" t="s">
-        <v>252</v>
+        <v>249</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="E4" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F4" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="B5" t="s">
-        <v>263</v>
-      </c>
-      <c r="C5" t="s">
         <v>252</v>
       </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
       <c r="D5" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="E5" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F5" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="B6" t="s">
-        <v>266</v>
-      </c>
-      <c r="C6" t="s">
-        <v>267</v>
+        <v>255</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E6" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F6" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="B7" t="s">
-        <v>269</v>
-      </c>
-      <c r="C7" t="s">
-        <v>267</v>
+        <v>257</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="E7" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F7" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="B8" t="s">
-        <v>271</v>
-      </c>
-      <c r="C8" t="s">
-        <v>252</v>
+        <v>259</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E8" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F8" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="B9" t="s">
-        <v>274</v>
-      </c>
-      <c r="C9" t="s">
-        <v>252</v>
+        <v>262</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="E9" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F9" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="B10" t="s">
-        <v>277</v>
-      </c>
-      <c r="C10" t="s">
-        <v>278</v>
+        <v>265</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>279</v>
+        <v>266</v>
       </c>
       <c r="E10" t="s">
-        <v>280</v>
+        <v>267</v>
       </c>
       <c r="F10" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>281</v>
+        <v>268</v>
       </c>
       <c r="B11" t="s">
-        <v>282</v>
-      </c>
-      <c r="C11" t="s">
-        <v>267</v>
+        <v>269</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
       <c r="E11" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F11" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
       <c r="B12" t="s">
-        <v>285</v>
-      </c>
-      <c r="C12" t="s">
-        <v>252</v>
+        <v>272</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="E12" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F12" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="B13" t="s">
-        <v>288</v>
-      </c>
-      <c r="C13" t="s">
-        <v>252</v>
+        <v>275</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
       </c>
       <c r="D13" t="s">
-        <v>289</v>
+        <v>276</v>
       </c>
       <c r="E13" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="F13" t="s">
-        <v>255</v>
+        <v>244</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>354</v>
+      </c>
+      <c r="B14" t="s">
+        <v>355</v>
+      </c>
+      <c r="C14" t="s">
+        <v>365</v>
+      </c>
+      <c r="D14" t="s">
+        <v>356</v>
+      </c>
+      <c r="E14" t="s">
+        <v>243</v>
+      </c>
+      <c r="F14" t="s">
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -3926,7 +4077,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -3934,252 +4085,275 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>290</v>
+        <v>277</v>
       </c>
       <c r="C1" t="s">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="D1" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E1" t="s">
-        <v>292</v>
+        <v>279</v>
       </c>
       <c r="F1" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="G1" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="B2" t="s">
-        <v>295</v>
+        <v>282</v>
       </c>
       <c r="C2" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D2" t="s">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="E2" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="F2" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G2" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>298</v>
+        <v>285</v>
       </c>
       <c r="B3" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="C3" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="D3" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="E3" t="s">
-        <v>301</v>
+        <v>288</v>
       </c>
       <c r="F3" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>302</v>
+        <v>289</v>
       </c>
       <c r="B4" t="s">
-        <v>303</v>
+        <v>290</v>
       </c>
       <c r="C4" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="D4" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
       <c r="E4" t="s">
-        <v>305</v>
+        <v>292</v>
       </c>
       <c r="F4" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G4" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="B5" t="s">
-        <v>307</v>
+        <v>294</v>
       </c>
       <c r="C5" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="D5" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
       <c r="E5" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="F5" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G5" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>309</v>
+        <v>296</v>
       </c>
       <c r="B6" t="s">
-        <v>310</v>
+        <v>297</v>
       </c>
       <c r="C6" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="D6" t="s">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="E6" t="s">
-        <v>311</v>
+        <v>298</v>
       </c>
       <c r="F6" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>312</v>
+        <v>299</v>
       </c>
       <c r="B7" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="C7" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="D7" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="E7" t="s">
-        <v>301</v>
+        <v>288</v>
       </c>
       <c r="F7" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="B8" t="s">
-        <v>315</v>
+        <v>302</v>
       </c>
       <c r="C8" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="D8" t="s">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="E8" t="s">
-        <v>316</v>
+        <v>303</v>
       </c>
       <c r="F8" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>317</v>
+        <v>304</v>
       </c>
       <c r="B9" t="s">
-        <v>318</v>
+        <v>305</v>
       </c>
       <c r="C9" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="D9" t="s">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="E9" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="F9" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
       <c r="B10" t="s">
-        <v>320</v>
+        <v>307</v>
       </c>
       <c r="C10" t="s">
-        <v>321</v>
+        <v>308</v>
       </c>
       <c r="D10" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
       <c r="E10" t="s">
-        <v>322</v>
+        <v>309</v>
       </c>
       <c r="F10" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G10" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>323</v>
+        <v>310</v>
       </c>
       <c r="B11" t="s">
-        <v>324</v>
+        <v>311</v>
       </c>
       <c r="C11" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="D11" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="E11" t="s">
-        <v>301</v>
+        <v>288</v>
       </c>
       <c r="F11" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="G11" t="s">
-        <v>28</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>366</v>
+      </c>
+      <c r="B12" t="s">
+        <v>358</v>
+      </c>
+      <c r="C12" t="s">
+        <v>308</v>
+      </c>
+      <c r="D12" t="s">
+        <v>359</v>
+      </c>
+      <c r="E12" t="s">
+        <v>360</v>
+      </c>
+      <c r="F12" t="s">
+        <v>284</v>
+      </c>
+      <c r="G12" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -4192,7 +4366,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -4203,73 +4377,84 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>325</v>
+        <v>312</v>
       </c>
       <c r="B2" t="s">
-        <v>326</v>
+        <v>313</v>
       </c>
       <c r="C2" t="s">
-        <v>327</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="B3" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
       <c r="C3" t="s">
-        <v>330</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="B4" t="s">
-        <v>332</v>
+        <v>319</v>
       </c>
       <c r="C4" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
       <c r="B5" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="C5" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
       <c r="B6" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="C6" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="B7" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
       <c r="C7" t="s">
-        <v>342</v>
+        <v>329</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>345</v>
+      </c>
+      <c r="B8" t="s">
+        <v>367</v>
+      </c>
+      <c r="C8" t="s">
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -4292,62 +4477,62 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>348</v>
+        <v>335</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>349</v>
+        <v>336</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>350</v>
+        <v>337</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>352</v>
+        <v>339</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>353</v>
+        <v>340</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>354</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: resolve blank page crash block by correctly parsing undefined Excel arrays and matching Creators schema properties
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xueruifang/Desktop/手搓我的Sims世界/sims-files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xueruifang/Desktop/手搓我的Sims世界/sims-files/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8354D9D-4B65-DE46-9552-205DC9957E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40951F2-54C4-3E4B-9DEB-166D11912C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sims" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: support uppercase image extensions in SmartImage
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xueruifang/Desktop/手搓我的Sims世界/sims-files/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B670166-63FD-E54E-8918-20AAEB4C39EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116B57E5-C8B4-EA46-B5A3-9FBE923D0323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="760" windowWidth="23640" windowHeight="18880" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6420" yWindow="760" windowWidth="23640" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worlds" sheetId="4" r:id="rId1"/>

</xml_diff>

<commit_message>
style: change district image aspect ratio to 3:2
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xueruifang/Desktop/手搓我的Sims世界/sims-files/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F156EB5E-A8FB-B943-A160-F60EB148AAAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78528BB9-4F77-EE4F-8CBA-DF62C543C22E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="760" windowWidth="23640" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6420" yWindow="760" windowWidth="23640" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worlds" sheetId="4" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="284">
   <si>
     <t>id</t>
   </si>
@@ -1744,7 +1744,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -1820,14 +1820,6 @@
         <v>180</v>
       </c>
       <c r="B7" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8" t="s">
         <v>283</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: simplify excel schema with lookup-based name resolution
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xueruifang/Desktop/手搓我的Sims世界/sims-files/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78528BB9-4F77-EE4F-8CBA-DF62C543C22E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E062268-4B3C-374D-BBE6-0D431A785AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="760" windowWidth="23640" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7460" yWindow="760" windowWidth="20480" windowHeight="18880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worlds" sheetId="4" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="263">
   <si>
     <t>id</t>
   </si>
@@ -135,15 +135,6 @@
     <t>Writing:8,Logic:6,Charisma:5</t>
   </si>
   <si>
-    <t>spencer-kim-lewis</t>
-  </si>
-  <si>
-    <t>pancakes</t>
-  </si>
-  <si>
-    <t>fangfang</t>
-  </si>
-  <si>
     <t>Oasis Springs</t>
   </si>
   <si>
@@ -168,99 +159,21 @@
     <t>The aristocrats of Willow Creek. Known for their gloomy demeanor and mysterious past, the Goths are staples of the community with secrets buried deep within their history.</t>
   </si>
   <si>
-    <t>ophelia-villa</t>
-  </si>
-  <si>
     <t>Spencer-Kim-Lewis</t>
   </si>
   <si>
-    <t>斯宾塞-金-刘易斯</t>
-  </si>
-  <si>
     <t>A modern blended family living in a large modern home. They represent the new generation of Willow Creek residents.</t>
   </si>
   <si>
-    <t>cypress-terrace</t>
-  </si>
-  <si>
     <t>Pancakes</t>
   </si>
   <si>
-    <t>bff</t>
-  </si>
-  <si>
-    <t>BFF Household</t>
-  </si>
-  <si>
-    <t>landgraab</t>
-  </si>
-  <si>
-    <t>Landgraab</t>
-  </si>
-  <si>
-    <t>caliente</t>
-  </si>
-  <si>
-    <t>Caliente</t>
-  </si>
-  <si>
-    <t>zest</t>
-  </si>
-  <si>
-    <t>Zest</t>
-  </si>
-  <si>
-    <t>roomies</t>
-  </si>
-  <si>
-    <t>Roomies</t>
-  </si>
-  <si>
-    <t>villareal</t>
-  </si>
-  <si>
-    <t>Villareal</t>
-  </si>
-  <si>
     <t>Windenburg</t>
   </si>
   <si>
-    <t>fyres</t>
-  </si>
-  <si>
-    <t>Fyres</t>
-  </si>
-  <si>
-    <t>bjergsen</t>
-  </si>
-  <si>
-    <t>Bjergsen</t>
-  </si>
-  <si>
-    <t>bro</t>
-  </si>
-  <si>
-    <t>Partihaus</t>
-  </si>
-  <si>
-    <t>karaoke</t>
-  </si>
-  <si>
-    <t>Karaoke Legends</t>
-  </si>
-  <si>
     <t>San Myshuno</t>
   </si>
   <si>
-    <t>pizza</t>
-  </si>
-  <si>
-    <t>Pizza Enthusiasts</t>
-  </si>
-  <si>
-    <t>FANGFFF</t>
-  </si>
-  <si>
     <t>size</t>
   </si>
   <si>
@@ -336,15 +249,6 @@
     <t>温登堡</t>
   </si>
   <si>
-    <t>A quiet, affordable neighborhood perfect for starters.</t>
-  </si>
-  <si>
-    <t>A charming middle-class area with larger homes.</t>
-  </si>
-  <si>
-    <t>The most prestigious address in Willow Creek.</t>
-  </si>
-  <si>
     <t>favLevel</t>
   </si>
   <si>
@@ -570,75 +474,12 @@
     <t>15x10</t>
   </si>
   <si>
-    <t>Willow-Creek</t>
-  </si>
-  <si>
-    <t>Foundry-Cove</t>
-  </si>
-  <si>
-    <t>Courtyard-Lane</t>
-  </si>
-  <si>
-    <t>Pendula-View</t>
-  </si>
-  <si>
-    <t>Sage-Estates</t>
-  </si>
-  <si>
-    <t>Crawdad-Quarter</t>
-  </si>
-  <si>
-    <t>Magnolia-Blossom-Park</t>
-  </si>
-  <si>
     <t>柳溪是一个郁郁葱葱的河口，连绵丘陵与沼泽水道在此交织难分。这里不仅有历久不衰的名声，也以充满了河岸人民好客精神的简朴生活风格闻名。柳溪有完善的城镇生活设施，活泼的邻居，以及各种资产可能性的宏大愿景，绝对是一个适合放松身心和落地生根的快乐无忧之地。</t>
   </si>
   <si>
-    <t>Oasis-Springs</t>
-  </si>
-  <si>
     <t>Forgotten Hollow</t>
   </si>
   <si>
-    <t>Magnolia-Promenade</t>
-  </si>
-  <si>
-    <t>San-Myshuno</t>
-  </si>
-  <si>
-    <t>Forgotten-Hollow</t>
-  </si>
-  <si>
-    <t>Brindleton-Bay</t>
-  </si>
-  <si>
-    <t>Del-Sol-Valley</t>
-  </si>
-  <si>
-    <t>Stranger-Ville</t>
-  </si>
-  <si>
-    <t>Evergreen-Harbor</t>
-  </si>
-  <si>
-    <t>Mt-Komorebi</t>
-  </si>
-  <si>
-    <t>Moonwood-Mill</t>
-  </si>
-  <si>
-    <t>San-Sequoia</t>
-  </si>
-  <si>
-    <t>Chestnut-Ridge</t>
-  </si>
-  <si>
-    <t>Ciudad-Enamorada</t>
-  </si>
-  <si>
-    <t>Gibbi-Point</t>
-  </si>
-  <si>
     <t>绿洲被西部沙漠的简朴之美所包围，这个兼容并蓄文化的天堂遍布无数高耸的棕榈树，郁郁葱葱的景观散发出鲜艳的色彩。绿洲之泉为任何发现它的旅人，提供躲避烈日的歇脚处。</t>
   </si>
   <si>
@@ -801,9 +642,6 @@
     <t>微光溪流这座小镇的内幕，也许不如表面上那般宁静…</t>
   </si>
   <si>
-    <t>Granite-Falls</t>
-  </si>
-  <si>
     <t>Residential</t>
   </si>
   <si>
@@ -825,74 +663,179 @@
     <t>Secret lot</t>
   </si>
   <si>
-    <t>Bargain-Bend</t>
-  </si>
-  <si>
-    <t>Streamlet-Single</t>
-  </si>
-  <si>
-    <t>Crick-Cabana</t>
-  </si>
-  <si>
-    <t>Daisy-Hovel</t>
-  </si>
-  <si>
-    <t>Garden-Essence</t>
-  </si>
-  <si>
-    <t>Potters-Splay</t>
-  </si>
-  <si>
-    <t>Brook-Bungalow</t>
-  </si>
-  <si>
-    <t>Riverside-Roost</t>
-  </si>
-  <si>
-    <t>Pique-Hearth</t>
-  </si>
-  <si>
-    <t>Rindle-Rose</t>
-  </si>
-  <si>
-    <t>Hallow-Slough</t>
-  </si>
-  <si>
-    <t>Umbrage-Manor</t>
-  </si>
-  <si>
-    <t>Ophelia-Villa</t>
-  </si>
-  <si>
-    <t>Cypress-Terrace</t>
-  </si>
-  <si>
-    <t>Municipal-Muses-Museum</t>
-  </si>
-  <si>
-    <t>The-Blue-Velvet-Nightclub</t>
-  </si>
-  <si>
-    <t>Movers-Shakers-Gym</t>
-  </si>
-  <si>
-    <t>Willow-Creek-Archive-Library</t>
-  </si>
-  <si>
-    <t>Sylvan-Glade</t>
+    <t>天井路</t>
+  </si>
+  <si>
+    <t>芳得利湾</t>
+  </si>
+  <si>
+    <t>花园社区</t>
+  </si>
+  <si>
+    <t>小龙虾区</t>
+  </si>
+  <si>
+    <t>贤者产业</t>
+  </si>
+  <si>
+    <t>林间空地</t>
+  </si>
+  <si>
+    <t>Goth</t>
+  </si>
+  <si>
+    <t>BFF</t>
+  </si>
+  <si>
+    <t>CypressTerrace</t>
+  </si>
+  <si>
+    <t>OpheliaVilla</t>
+  </si>
+  <si>
+    <t>CourtyardLane</t>
+  </si>
+  <si>
+    <t>GardenEssence</t>
+  </si>
+  <si>
+    <t>WillowCreek</t>
+  </si>
+  <si>
+    <t>OasisSprings</t>
+  </si>
+  <si>
+    <t>GraniteFalls</t>
+  </si>
+  <si>
+    <t>MagnoliaPromenade</t>
+  </si>
+  <si>
+    <t>SanMyshuno</t>
+  </si>
+  <si>
+    <t>ForgottenHollow</t>
+  </si>
+  <si>
+    <t>BrindletonBay</t>
+  </si>
+  <si>
+    <t>DelSolValley</t>
+  </si>
+  <si>
+    <t>StrangerVille</t>
+  </si>
+  <si>
+    <t>EvergreenHarbor</t>
+  </si>
+  <si>
+    <t>MtKomorebi</t>
+  </si>
+  <si>
+    <t>HenfordOnBagley</t>
+  </si>
+  <si>
+    <t>MoonwoodMill</t>
+  </si>
+  <si>
+    <t>SanSequoia</t>
+  </si>
+  <si>
+    <t>ChestnutRidge</t>
+  </si>
+  <si>
+    <t>CiudadEnamorada</t>
+  </si>
+  <si>
+    <t>GibbiPoint</t>
+  </si>
+  <si>
+    <t>FoundryCove</t>
+  </si>
+  <si>
+    <t>PendulaView</t>
+  </si>
+  <si>
+    <t>SageEstates</t>
+  </si>
+  <si>
+    <t>CrawdadQuarter</t>
+  </si>
+  <si>
+    <t>SylvanGlade</t>
+  </si>
+  <si>
+    <t>BargainBend</t>
+  </si>
+  <si>
+    <t>StreamletSingle</t>
+  </si>
+  <si>
+    <t>CrickCabana</t>
+  </si>
+  <si>
+    <t>DaisyHovel</t>
+  </si>
+  <si>
+    <t>PottersSplay</t>
+  </si>
+  <si>
+    <t>BrookBungalow</t>
+  </si>
+  <si>
+    <t>RiversideRoost</t>
+  </si>
+  <si>
+    <t>PiqueHearth</t>
+  </si>
+  <si>
+    <t>RindleRose</t>
+  </si>
+  <si>
+    <t>HallowSlough</t>
+  </si>
+  <si>
+    <t>UmbrageManor</t>
+  </si>
+  <si>
+    <t>MunicipalMusesMuseum</t>
+  </si>
+  <si>
+    <t>TheBlueVelvetNightclub</t>
+  </si>
+  <si>
+    <t>MoversShakersGym</t>
+  </si>
+  <si>
+    <t>WillowCreekArchiveLibrary</t>
+  </si>
+  <si>
+    <t>MagnoliaBlossomPark</t>
+  </si>
+  <si>
+    <t>SpencerKimLewis</t>
+  </si>
+  <si>
+    <t>斯宾塞-金-路易斯</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF404040"/>
+      <name val="Trebuchet MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -927,13 +870,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1292,449 +1236,449 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E1" t="s">
-        <v>94</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B2" t="s">
         <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>187</v>
+        <v>148</v>
       </c>
       <c r="E2" t="s">
-        <v>96</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>188</v>
+        <v>224</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="D3" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="E3" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
-        <v>204</v>
+        <v>151</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>108</v>
       </c>
       <c r="C5" t="s">
-        <v>255</v>
+        <v>202</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>190</v>
+        <v>226</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
-        <v>206</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>205</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>207</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>191</v>
+        <v>227</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>192</v>
+        <v>228</v>
       </c>
       <c r="B9" t="s">
-        <v>189</v>
+        <v>149</v>
       </c>
       <c r="C9" t="s">
-        <v>210</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>209</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>193</v>
+        <v>229</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>110</v>
       </c>
       <c r="C10" t="s">
-        <v>212</v>
+        <v>159</v>
       </c>
       <c r="D10" t="s">
-        <v>211</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>143</v>
+        <v>111</v>
       </c>
       <c r="B11" t="s">
-        <v>143</v>
+        <v>111</v>
       </c>
       <c r="C11" t="s">
-        <v>213</v>
+        <v>160</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>194</v>
+        <v>230</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="C12" t="s">
-        <v>215</v>
+        <v>162</v>
       </c>
       <c r="D12" t="s">
-        <v>214</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>195</v>
+        <v>231</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>217</v>
+        <v>164</v>
       </c>
       <c r="D13" t="s">
-        <v>216</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="C14" t="s">
-        <v>219</v>
+        <v>166</v>
       </c>
       <c r="D14" t="s">
-        <v>218</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
-        <v>222</v>
+        <v>169</v>
       </c>
       <c r="D15" t="s">
-        <v>256</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="B16" t="s">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="C16" t="s">
-        <v>221</v>
+        <v>168</v>
       </c>
       <c r="D16" t="s">
-        <v>220</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>196</v>
+        <v>232</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="C17" t="s">
-        <v>224</v>
+        <v>171</v>
       </c>
       <c r="D17" t="s">
-        <v>223</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>150</v>
+        <v>118</v>
       </c>
       <c r="B18" t="s">
-        <v>150</v>
+        <v>118</v>
       </c>
       <c r="C18" t="s">
-        <v>226</v>
+        <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>225</v>
+        <v>172</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>197</v>
+        <v>233</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>119</v>
       </c>
       <c r="C19" t="s">
-        <v>228</v>
+        <v>175</v>
       </c>
       <c r="D19" t="s">
-        <v>227</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>152</v>
+        <v>234</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>120</v>
       </c>
       <c r="C20" t="s">
-        <v>230</v>
+        <v>177</v>
       </c>
       <c r="D20" t="s">
-        <v>229</v>
+        <v>176</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="C21" t="s">
-        <v>232</v>
+        <v>179</v>
       </c>
       <c r="D21" t="s">
-        <v>231</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>198</v>
+        <v>235</v>
       </c>
       <c r="B22" t="s">
-        <v>154</v>
+        <v>122</v>
       </c>
       <c r="C22" t="s">
-        <v>236</v>
+        <v>183</v>
       </c>
       <c r="D22" t="s">
-        <v>235</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>155</v>
+        <v>123</v>
       </c>
       <c r="B23" t="s">
-        <v>155</v>
+        <v>123</v>
       </c>
       <c r="C23" t="s">
-        <v>234</v>
+        <v>181</v>
       </c>
       <c r="D23" t="s">
-        <v>233</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>199</v>
+        <v>236</v>
       </c>
       <c r="B24" t="s">
-        <v>156</v>
+        <v>124</v>
       </c>
       <c r="C24" t="s">
-        <v>238</v>
+        <v>185</v>
       </c>
       <c r="D24" t="s">
-        <v>237</v>
+        <v>184</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>200</v>
+        <v>237</v>
       </c>
       <c r="B25" t="s">
-        <v>157</v>
+        <v>125</v>
       </c>
       <c r="C25" t="s">
-        <v>240</v>
+        <v>187</v>
       </c>
       <c r="D25" t="s">
-        <v>239</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>158</v>
+        <v>126</v>
       </c>
       <c r="B26" t="s">
-        <v>158</v>
+        <v>126</v>
       </c>
       <c r="C26" t="s">
-        <v>242</v>
+        <v>189</v>
       </c>
       <c r="D26" t="s">
-        <v>241</v>
+        <v>188</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>201</v>
+        <v>238</v>
       </c>
       <c r="B27" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="C27" t="s">
-        <v>244</v>
+        <v>191</v>
       </c>
       <c r="D27" t="s">
-        <v>243</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="C28" t="s">
-        <v>246</v>
+        <v>193</v>
       </c>
       <c r="D28" t="s">
-        <v>245</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>161</v>
+        <v>129</v>
       </c>
       <c r="B29" t="s">
-        <v>161</v>
+        <v>129</v>
       </c>
       <c r="C29" t="s">
-        <v>248</v>
+        <v>195</v>
       </c>
       <c r="D29" t="s">
-        <v>247</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="B30" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="C30" t="s">
-        <v>250</v>
+        <v>197</v>
       </c>
       <c r="D30" t="s">
-        <v>249</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>202</v>
+        <v>239</v>
       </c>
       <c r="B31" t="s">
-        <v>163</v>
+        <v>131</v>
       </c>
       <c r="C31" t="s">
-        <v>252</v>
+        <v>199</v>
       </c>
       <c r="D31" t="s">
-        <v>251</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>164</v>
+        <v>132</v>
       </c>
       <c r="B32" t="s">
-        <v>164</v>
+        <v>132</v>
       </c>
       <c r="C32" t="s">
-        <v>254</v>
+        <v>201</v>
       </c>
       <c r="D32" t="s">
-        <v>253</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -1763,70 +1707,79 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D2" t="s">
-        <v>102</v>
+        <v>240</v>
+      </c>
+      <c r="C2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B3" t="s">
-        <v>182</v>
-      </c>
-      <c r="D3" t="s">
-        <v>103</v>
+        <v>221</v>
+      </c>
+      <c r="C3" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B4" t="s">
-        <v>183</v>
+        <v>241</v>
+      </c>
+      <c r="C4" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B5" t="s">
-        <v>184</v>
-      </c>
-      <c r="D5" t="s">
-        <v>104</v>
+        <v>242</v>
+      </c>
+      <c r="C5" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B6" t="s">
-        <v>185</v>
+        <v>243</v>
+      </c>
+      <c r="C6" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B7" t="s">
-        <v>283</v>
+        <v>244</v>
+      </c>
+      <c r="C7" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 D5 D2:D3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1838,6 +1791,7 @@
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="27.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" customWidth="1"/>
     <col min="6" max="6" width="19.33203125" customWidth="1"/>
     <col min="7" max="7" width="10.33203125" customWidth="1"/>
@@ -1854,45 +1808,45 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="E1" t="s">
         <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="H1" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="I1" t="s">
-        <v>81</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="B2" t="s">
-        <v>165</v>
+        <v>133</v>
       </c>
       <c r="C2" t="s">
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E2" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F2" t="s">
-        <v>181</v>
+        <v>240</v>
       </c>
       <c r="G2" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="H2" t="s">
         <v>32</v>
@@ -1903,22 +1857,22 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>167</v>
+        <v>135</v>
       </c>
       <c r="E3" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F3" t="s">
-        <v>181</v>
+        <v>240</v>
       </c>
       <c r="G3" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I3" t="s">
         <v>31</v>
@@ -1926,22 +1880,22 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>167</v>
+        <v>135</v>
       </c>
       <c r="E4" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F4" t="s">
-        <v>181</v>
+        <v>240</v>
       </c>
       <c r="G4" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I4" t="s">
         <v>31</v>
@@ -1949,22 +1903,22 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>54</v>
       </c>
       <c r="D5" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E5" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F5" t="s">
-        <v>181</v>
+        <v>240</v>
       </c>
       <c r="G5" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I5" t="s">
         <v>31</v>
@@ -1972,22 +1926,22 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>269</v>
+        <v>222</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="D6" t="s">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="E6" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F6" t="s">
-        <v>181</v>
+        <v>240</v>
       </c>
       <c r="G6" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I6" t="s">
         <v>31</v>
@@ -1995,22 +1949,22 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E7" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F7" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="G7" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I7" t="s">
         <v>31</v>
@@ -2018,22 +1972,22 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="D8" t="s">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="E8" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F8" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="G8" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I8" t="s">
         <v>31</v>
@@ -2041,22 +1995,22 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E9" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F9" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="G9" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I9" t="s">
         <v>31</v>
@@ -2064,22 +2018,22 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="B10" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D10" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F10" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="G10" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I10" t="s">
         <v>31</v>
@@ -2087,22 +2041,22 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>274</v>
+        <v>253</v>
       </c>
       <c r="B11" t="s">
-        <v>170</v>
+        <v>138</v>
       </c>
       <c r="D11" t="s">
-        <v>167</v>
+        <v>135</v>
       </c>
       <c r="E11" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F11" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="G11" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I11" t="s">
         <v>31</v>
@@ -2110,22 +2064,22 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>275</v>
+        <v>254</v>
       </c>
       <c r="B12" t="s">
-        <v>171</v>
+        <v>139</v>
       </c>
       <c r="D12" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E12" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F12" t="s">
-        <v>183</v>
+        <v>241</v>
       </c>
       <c r="G12" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I12" t="s">
         <v>31</v>
@@ -2133,22 +2087,22 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>276</v>
+        <v>255</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="E13" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F13" t="s">
-        <v>183</v>
+        <v>241</v>
       </c>
       <c r="G13" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I13" t="s">
         <v>31</v>
@@ -2156,22 +2110,22 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>172</v>
+        <v>140</v>
       </c>
       <c r="B14" t="s">
-        <v>172</v>
+        <v>140</v>
       </c>
       <c r="D14" t="s">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="E14" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F14" t="s">
-        <v>183</v>
+        <v>241</v>
       </c>
       <c r="G14" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I14" t="s">
         <v>31</v>
@@ -2179,22 +2133,22 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>277</v>
+        <v>220</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E15" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F15" t="s">
-        <v>183</v>
+        <v>241</v>
       </c>
       <c r="G15" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I15" t="s">
         <v>31</v>
@@ -2202,22 +2156,22 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
       <c r="B16" t="s">
-        <v>173</v>
+        <v>141</v>
       </c>
       <c r="D16" t="s">
-        <v>174</v>
+        <v>142</v>
       </c>
       <c r="E16" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F16" t="s">
-        <v>184</v>
+        <v>242</v>
       </c>
       <c r="G16" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I16" t="s">
         <v>31</v>
@@ -2225,22 +2179,22 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>278</v>
+        <v>219</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="D17" t="s">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="E17" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F17" t="s">
-        <v>184</v>
+        <v>242</v>
       </c>
       <c r="G17" t="s">
-        <v>258</v>
+        <v>204</v>
       </c>
       <c r="I17" t="s">
         <v>31</v>
@@ -2248,22 +2202,22 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>279</v>
+        <v>256</v>
       </c>
       <c r="B18" t="s">
-        <v>175</v>
+        <v>143</v>
       </c>
       <c r="D18" t="s">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="E18" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F18" t="s">
-        <v>185</v>
+        <v>243</v>
       </c>
       <c r="G18" t="s">
-        <v>259</v>
+        <v>205</v>
       </c>
       <c r="I18" t="s">
         <v>31</v>
@@ -2271,22 +2225,22 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>280</v>
+        <v>257</v>
       </c>
       <c r="B19" t="s">
-        <v>176</v>
+        <v>144</v>
       </c>
       <c r="D19" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E19" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F19" t="s">
-        <v>185</v>
+        <v>243</v>
       </c>
       <c r="G19" t="s">
-        <v>260</v>
+        <v>206</v>
       </c>
       <c r="I19" t="s">
         <v>31</v>
@@ -2294,22 +2248,22 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>281</v>
+        <v>258</v>
       </c>
       <c r="B20" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D20" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E20" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F20" t="s">
-        <v>185</v>
+        <v>243</v>
       </c>
       <c r="G20" t="s">
-        <v>261</v>
+        <v>207</v>
       </c>
       <c r="I20" t="s">
         <v>31</v>
@@ -2317,22 +2271,22 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>282</v>
+        <v>259</v>
       </c>
       <c r="B21" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="D21" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="E21" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F21" t="s">
-        <v>185</v>
+        <v>243</v>
       </c>
       <c r="G21" t="s">
-        <v>262</v>
+        <v>208</v>
       </c>
       <c r="I21" t="s">
         <v>31</v>
@@ -2340,22 +2294,22 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>186</v>
+        <v>260</v>
       </c>
       <c r="B22" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>174</v>
+        <v>142</v>
       </c>
       <c r="E22" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F22" t="s">
-        <v>185</v>
+        <v>243</v>
       </c>
       <c r="G22" t="s">
-        <v>263</v>
+        <v>209</v>
       </c>
       <c r="I22" t="s">
         <v>31</v>
@@ -2363,22 +2317,22 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>283</v>
+        <v>244</v>
       </c>
       <c r="B23" t="s">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="D23" t="s">
-        <v>179</v>
+        <v>147</v>
       </c>
       <c r="E23" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="F23" t="s">
-        <v>283</v>
+        <v>244</v>
       </c>
       <c r="G23" t="s">
-        <v>264</v>
+        <v>210</v>
       </c>
       <c r="I23" t="s">
         <v>31</v>
@@ -2394,8 +2348,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="26.5" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -2408,7 +2367,7 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E1" t="s">
         <v>7</v>
@@ -2417,409 +2376,99 @@
         <v>8</v>
       </c>
       <c r="G1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B2" t="s">
         <v>40</v>
       </c>
-      <c r="H1" t="s">
+      <c r="C2" t="s">
         <v>41</v>
       </c>
-      <c r="I1" t="s">
+      <c r="D2" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" t="s">
-        <v>45</v>
       </c>
       <c r="E2" t="s">
         <v>28</v>
       </c>
+      <c r="F2" t="s">
+        <v>223</v>
+      </c>
       <c r="G2" t="s">
         <v>32</v>
       </c>
       <c r="H2" t="s">
-        <v>46</v>
+        <v>220</v>
       </c>
       <c r="I2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>35</v>
+    <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>261</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>262</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
         <v>28</v>
       </c>
+      <c r="F3" t="s">
+        <v>223</v>
+      </c>
       <c r="G3" t="s">
         <v>32</v>
       </c>
-      <c r="H3" t="s">
-        <v>50</v>
+      <c r="H3" s="4" t="s">
+        <v>219</v>
       </c>
       <c r="I3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
+    <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" t="s">
+        <v>223</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="F5" t="s">
+        <v>223</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H7" t="s">
-        <v>32</v>
-      </c>
-      <c r="I7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" t="s">
-        <v>32</v>
-      </c>
-      <c r="I8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" t="s">
-        <v>32</v>
-      </c>
-      <c r="I9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" t="s">
-        <v>32</v>
-      </c>
-      <c r="I10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G11" t="s">
-        <v>32</v>
-      </c>
-      <c r="H11" t="s">
-        <v>32</v>
-      </c>
-      <c r="I11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>67</v>
-      </c>
-      <c r="B12" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" t="s">
-        <v>64</v>
-      </c>
-      <c r="G12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" t="s">
-        <v>32</v>
-      </c>
-      <c r="H13" t="s">
-        <v>32</v>
-      </c>
-      <c r="I13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B14" t="s">
-        <v>72</v>
-      </c>
-      <c r="C14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" t="s">
-        <v>73</v>
-      </c>
-      <c r="G14" t="s">
-        <v>32</v>
-      </c>
-      <c r="H14" t="s">
-        <v>32</v>
-      </c>
-      <c r="I14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" t="s">
-        <v>73</v>
-      </c>
-      <c r="G15" t="s">
-        <v>32</v>
-      </c>
-      <c r="H15" t="s">
-        <v>32</v>
-      </c>
-      <c r="I15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E16" t="s">
-        <v>73</v>
-      </c>
-      <c r="G16" t="s">
-        <v>32</v>
-      </c>
-      <c r="H16" t="s">
-        <v>32</v>
-      </c>
-      <c r="I16" t="s">
-        <v>32</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I16" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I1 B3 B2:D2 I2 I3 D3:E3 G2 G3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3190,36 +2839,36 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>105</v>
+        <v>73</v>
       </c>
       <c r="D1" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="E1" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="F1" t="s">
-        <v>108</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -3240,45 +2889,45 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>115</v>
+        <v>83</v>
       </c>
       <c r="C1" t="s">
-        <v>116</v>
+        <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="E1" t="s">
-        <v>117</v>
+        <v>85</v>
       </c>
       <c r="F1" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="G1" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
-        <v>121</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="F2" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
       <c r="G2" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -3302,18 +2951,18 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>108</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -3336,62 +2985,62 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>127</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>130</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>131</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>133</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>134</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>135</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>137</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>